<commit_message>
changed shop checking, cleaned up some code, added new main file
</commit_message>
<xml_diff>
--- a/config.xlsx
+++ b/config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10911"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kimbogyeong/Documents/GitHub/ETL/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://smu-my.sharepoint.com/personal/keithtan_2022_accountancy_smu_edu_sg/Documents/Desktop/smu/subject/y4s2/capstone/ETL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E3D9085-F648-3F49-90D7-93E0492F6F71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{6E3D9085-F648-3F49-90D7-93E0492F6F71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D87C2FDF-5E5D-4054-AFD6-E70A8E73CA72}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="paths" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
   <si>
     <t>raw_data</t>
   </si>
@@ -71,6 +71,9 @@
   </si>
   <si>
     <t>/Users/kimbogyeong/Desktop/Capstone/raw data</t>
+  </si>
+  <si>
+    <t>combined_data</t>
   </si>
 </sst>
 </file>
@@ -86,12 +89,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -106,8 +115,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -388,13 +398,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -402,7 +412,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -410,7 +420,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -418,11 +428,17 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="1"/>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>2</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B5" t="s">
         <v>12</v>
       </c>
     </row>
@@ -434,14 +450,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9EF9E44-D244-4891-A14F-02851A432852}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.1640625" customWidth="1"/>
+    <col min="1" max="1" width="15.140625" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="15.5" customWidth="1"/>
+    <col min="3" max="3" width="15.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -452,7 +468,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -463,7 +479,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -474,7 +490,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>

</xml_diff>